<commit_message>
fix: default date state in Checkout.jsx and robust React value setter in checkout.page.js
</commit_message>
<xml_diff>
--- a/excel/E2E_Report.xlsx
+++ b/excel/E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="111">
   <si>
     <t>Execution Date</t>
   </si>
@@ -40,7 +40,7 @@
     <t>Execution Duration (ms)</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:09 AM</t>
+    <t>7/23/2026, 10:15:00 AM</t>
   </si>
   <si>
     <t>Development</t>
@@ -85,10 +85,10 @@
     <t>Chrome</t>
   </si>
   <si>
-    <t>7/23/2026, 9:52:49 AM</t>
-  </si>
-  <si>
-    <t>7/23/2026, 9:52:54 AM</t>
+    <t>7/23/2026, 10:14:44 AM</t>
+  </si>
+  <si>
+    <t>7/23/2026, 10:14:49 AM</t>
   </si>
   <si>
     <t>TC-CORE-002</t>
@@ -97,7 +97,7 @@
     <t>Should register a new caterer</t>
   </si>
   <si>
-    <t>7/23/2026, 9:52:55 AM</t>
+    <t>7/23/2026, 10:14:50 AM</t>
   </si>
   <si>
     <t>TC-CORE-003</t>
@@ -106,7 +106,7 @@
     <t>Should login as admin and approve the pending caterer</t>
   </si>
   <si>
-    <t>7/23/2026, 9:52:56 AM</t>
+    <t>7/23/2026, 10:14:52 AM</t>
   </si>
   <si>
     <t>TC-CORE-004</t>
@@ -115,7 +115,7 @@
     <t>Should login as customer, search, select menu, checkout and confirm booking request</t>
   </si>
   <si>
-    <t>7/23/2026, 9:52:58 AM</t>
+    <t>7/23/2026, 10:14:54 AM</t>
   </si>
   <si>
     <t>TC-DYN-001</t>
@@ -127,16 +127,13 @@
     <t>Validate authentication with empty email [TC-DYN-001]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:52:59 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-002</t>
   </si>
   <si>
     <t>Validate authentication with empty password [TC-DYN-002]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:00 AM</t>
+    <t>7/23/2026, 10:14:55 AM</t>
   </si>
   <si>
     <t>TC-DYN-003</t>
@@ -145,16 +142,13 @@
     <t>Validate authentication with invalid email format [TC-DYN-003]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:01 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-004</t>
   </si>
   <si>
     <t>Validate event guest count constraint under min limit (50) [TC-DYN-004]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:02 AM</t>
+    <t>7/23/2026, 10:14:56 AM</t>
   </si>
   <si>
     <t>TC-DYN-005</t>
@@ -163,7 +157,7 @@
     <t>Validate required constraint on field of type number in Checkout [TC-DYN-005]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:03 AM</t>
+    <t>7/23/2026, 10:14:57 AM</t>
   </si>
   <si>
     <t>TC-DYN-006</t>
@@ -172,33 +166,27 @@
     <t>Validate required constraint on field of type date in Checkout [TC-DYN-006]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:04 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-007</t>
   </si>
   <si>
     <t>Validate required constraint on field of type email in Login [TC-DYN-007]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:05 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-008</t>
   </si>
   <si>
     <t>Validate required constraint on field of type password in Login [TC-DYN-008]</t>
   </si>
   <si>
+    <t>7/23/2026, 10:14:58 AM</t>
+  </si>
+  <si>
     <t>TC-DYN-009</t>
   </si>
   <si>
     <t>Validate required constraint on field of type text in RegisterCaterer [TC-DYN-009]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:06 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-010</t>
   </si>
   <si>
@@ -211,7 +199,7 @@
     <t>Validate required constraint on field of type file in RegisterCaterer [TC-DYN-011]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:07 AM</t>
+    <t>7/23/2026, 10:14:59 AM</t>
   </si>
   <si>
     <t>TC-DYN-012</t>
@@ -226,9 +214,6 @@
     <t>Validate required constraint on field of type text in RegisterCustomer [TC-DYN-013]</t>
   </si>
   <si>
-    <t>7/23/2026, 9:53:08 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-014</t>
   </si>
   <si>
@@ -265,7 +250,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-07-23T04:22:49.654Z</t>
+    <t>2026-07-23T04:44:44.788Z</t>
   </si>
   <si>
     <t>Test Scenario Initiated</t>
@@ -274,7 +259,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-07-23T04:22:54.498Z</t>
+    <t>2026-07-23T04:44:49.492Z</t>
   </si>
   <si>
     <t>Test Scenario Completed</t>
@@ -283,97 +268,85 @@
     <t>Executed successfully</t>
   </si>
   <si>
-    <t>2026-07-23T04:22:54.499Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:22:55.748Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:22:56.720Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:22:58.975Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:22:58.976Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:22:59.697Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:22:59.698Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:00.490Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:00.491Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:01.571Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:02.661Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:02.662Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:03.566Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:04.368Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:04.369Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:05.041Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:05.044Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:05.519Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:05.520Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:06.055Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:06.056Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:06.650Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:06.652Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:07.192Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:07.607Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:07.608Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:08.207Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:08.208Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:08.760Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:08.761Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:23:09.248Z</t>
+    <t>2026-07-23T04:44:49.494Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:50.980Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:52.083Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:52.084Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:54.158Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:54.160Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:54.699Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:54.700Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:55.386Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:55.387Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:55.827Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:56.484Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:57.033Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:57.034Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:57.573Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:57.932Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:58.199Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:58.200Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:58.573Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:58.574Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:58.885Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:58.886Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:59.221Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:59.539Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:44:59.842Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:45:00.345Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:45:00.640Z</t>
   </si>
 </sst>
 </file>
@@ -874,7 +847,7 @@
         <v>10</v>
       </c>
       <c r="H2" s="2">
-        <v>19587</v>
+        <v>15851</v>
       </c>
     </row>
   </sheetData>
@@ -945,7 +918,7 @@
         <v>24</v>
       </c>
       <c r="H2" s="2">
-        <v>4845</v>
+        <v>4706</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -971,7 +944,7 @@
         <v>27</v>
       </c>
       <c r="H3" s="2">
-        <v>1250</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -997,7 +970,7 @@
         <v>30</v>
       </c>
       <c r="H4" s="2">
-        <v>972</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1023,7 +996,7 @@
         <v>33</v>
       </c>
       <c r="H5" s="2">
-        <v>2255</v>
+        <v>2075</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1046,21 +1019,21 @@
         <v>33</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="H6" s="2">
-        <v>721</v>
+        <v>540</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>22</v>
@@ -1069,24 +1042,24 @@
         <v>3</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H7" s="2">
-        <v>793</v>
+        <v>686</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>22</v>
@@ -1095,24 +1068,24 @@
         <v>3</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H8" s="2">
-        <v>1079</v>
+        <v>441</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>22</v>
@@ -1121,24 +1094,24 @@
         <v>3</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H9" s="2">
-        <v>1090</v>
+        <v>657</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>22</v>
@@ -1147,24 +1120,24 @@
         <v>3</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H10" s="2">
-        <v>905</v>
+        <v>549</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>22</v>
@@ -1173,24 +1146,24 @@
         <v>3</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H11" s="2">
-        <v>802</v>
+        <v>540</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>22</v>
@@ -1199,24 +1172,24 @@
         <v>3</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="H12" s="2">
-        <v>673</v>
+        <v>359</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>22</v>
@@ -1225,24 +1198,24 @@
         <v>3</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H13" s="2">
-        <v>477</v>
+        <v>267</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>22</v>
@@ -1251,24 +1224,24 @@
         <v>3</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H14" s="2">
-        <v>536</v>
+        <v>374</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>22</v>
@@ -1277,24 +1250,24 @@
         <v>3</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H15" s="2">
-        <v>594</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>22</v>
@@ -1303,24 +1276,24 @@
         <v>3</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="H16" s="2">
-        <v>541</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>22</v>
@@ -1329,24 +1302,24 @@
         <v>3</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="H17" s="2">
-        <v>415</v>
+        <v>318</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>22</v>
@@ -1355,24 +1328,24 @@
         <v>3</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="H18" s="2">
-        <v>599</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>22</v>
@@ -1381,24 +1354,24 @@
         <v>3</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="H19" s="2">
-        <v>553</v>
+        <v>503</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>22</v>
@@ -1407,13 +1380,13 @@
         <v>3</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H20" s="2">
-        <v>487</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -1435,19 +1408,19 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1470,665 +1443,665 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Chrome options window-size 1280x1024 for headless Linux runner
</commit_message>
<xml_diff>
--- a/excel/E2E_Report.xlsx
+++ b/excel/E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="121">
   <si>
     <t>Execution Date</t>
   </si>
@@ -40,7 +40,7 @@
     <t>Execution Duration (ms)</t>
   </si>
   <si>
-    <t>7/23/2026, 10:15:00 AM</t>
+    <t>7/23/2026, 10:21:28 AM</t>
   </si>
   <si>
     <t>Development</t>
@@ -85,10 +85,10 @@
     <t>Chrome</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:44 AM</t>
-  </si>
-  <si>
-    <t>7/23/2026, 10:14:49 AM</t>
+    <t>7/23/2026, 10:21:03 AM</t>
+  </si>
+  <si>
+    <t>7/23/2026, 10:21:09 AM</t>
   </si>
   <si>
     <t>TC-CORE-002</t>
@@ -97,7 +97,7 @@
     <t>Should register a new caterer</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:50 AM</t>
+    <t>7/23/2026, 10:21:10 AM</t>
   </si>
   <si>
     <t>TC-CORE-003</t>
@@ -106,7 +106,7 @@
     <t>Should login as admin and approve the pending caterer</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:52 AM</t>
+    <t>7/23/2026, 10:21:12 AM</t>
   </si>
   <si>
     <t>TC-CORE-004</t>
@@ -115,7 +115,7 @@
     <t>Should login as customer, search, select menu, checkout and confirm booking request</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:54 AM</t>
+    <t>7/23/2026, 10:21:16 AM</t>
   </si>
   <si>
     <t>TC-DYN-001</t>
@@ -127,13 +127,16 @@
     <t>Validate authentication with empty email [TC-DYN-001]</t>
   </si>
   <si>
+    <t>7/23/2026, 10:21:18 AM</t>
+  </si>
+  <si>
     <t>TC-DYN-002</t>
   </si>
   <si>
     <t>Validate authentication with empty password [TC-DYN-002]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:55 AM</t>
+    <t>7/23/2026, 10:21:19 AM</t>
   </si>
   <si>
     <t>TC-DYN-003</t>
@@ -142,13 +145,16 @@
     <t>Validate authentication with invalid email format [TC-DYN-003]</t>
   </si>
   <si>
+    <t>7/23/2026, 10:21:20 AM</t>
+  </si>
+  <si>
     <t>TC-DYN-004</t>
   </si>
   <si>
     <t>Validate event guest count constraint under min limit (50) [TC-DYN-004]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:56 AM</t>
+    <t>7/23/2026, 10:21:22 AM</t>
   </si>
   <si>
     <t>TC-DYN-005</t>
@@ -157,7 +163,7 @@
     <t>Validate required constraint on field of type number in Checkout [TC-DYN-005]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:57 AM</t>
+    <t>7/23/2026, 10:21:23 AM</t>
   </si>
   <si>
     <t>TC-DYN-006</t>
@@ -166,6 +172,9 @@
     <t>Validate required constraint on field of type date in Checkout [TC-DYN-006]</t>
   </si>
   <si>
+    <t>7/23/2026, 10:21:24 AM</t>
+  </si>
+  <si>
     <t>TC-DYN-007</t>
   </si>
   <si>
@@ -178,7 +187,7 @@
     <t>Validate required constraint on field of type password in Login [TC-DYN-008]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:58 AM</t>
+    <t>7/23/2026, 10:21:25 AM</t>
   </si>
   <si>
     <t>TC-DYN-009</t>
@@ -187,6 +196,9 @@
     <t>Validate required constraint on field of type text in RegisterCaterer [TC-DYN-009]</t>
   </si>
   <si>
+    <t>7/23/2026, 10:21:26 AM</t>
+  </si>
+  <si>
     <t>TC-DYN-010</t>
   </si>
   <si>
@@ -199,15 +211,15 @@
     <t>Validate required constraint on field of type file in RegisterCaterer [TC-DYN-011]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:14:59 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-012</t>
   </si>
   <si>
     <t>Validate required constraint on field of type password in RegisterCaterer [TC-DYN-012]</t>
   </si>
   <si>
+    <t>7/23/2026, 10:21:27 AM</t>
+  </si>
+  <si>
     <t>TC-DYN-013</t>
   </si>
   <si>
@@ -250,7 +262,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-07-23T04:44:44.788Z</t>
+    <t>2026-07-23T04:51:03.556Z</t>
   </si>
   <si>
     <t>Test Scenario Initiated</t>
@@ -259,7 +271,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-07-23T04:44:49.492Z</t>
+    <t>2026-07-23T04:51:09.169Z</t>
   </si>
   <si>
     <t>Test Scenario Completed</t>
@@ -268,85 +280,103 @@
     <t>Executed successfully</t>
   </si>
   <si>
-    <t>2026-07-23T04:44:49.494Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:50.980Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:52.083Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:52.084Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:54.158Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:54.160Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:54.699Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:54.700Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:55.386Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:55.387Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:55.827Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:56.484Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:57.033Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:57.034Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:57.573Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:57.932Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:58.199Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:58.200Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:58.573Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:58.574Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:58.885Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:58.886Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:59.221Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:59.539Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:44:59.842Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:45:00.345Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:45:00.640Z</t>
+    <t>2026-07-23T04:51:09.170Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:10.628Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:10.631Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:12.740Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:12.742Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:16.928Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:16.932Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:18.482Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:18.484Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:19.795Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:19.796Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:20.772Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:20.774Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:22.069Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:22.070Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:23.292Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:23.293Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:24.401Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:24.902Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:24.903Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:25.475Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:26.009Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:26.010Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:26.567Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:26.568Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:26.979Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:27.358Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:27.359Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:27.821Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:27.822Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:28.304Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:28.305Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T04:51:28.762Z</t>
   </si>
 </sst>
 </file>
@@ -847,7 +877,7 @@
         <v>10</v>
       </c>
       <c r="H2" s="2">
-        <v>15851</v>
+        <v>25192</v>
       </c>
     </row>
   </sheetData>
@@ -918,7 +948,7 @@
         <v>24</v>
       </c>
       <c r="H2" s="2">
-        <v>4706</v>
+        <v>5614</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -944,7 +974,7 @@
         <v>27</v>
       </c>
       <c r="H3" s="2">
-        <v>1487</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -970,7 +1000,7 @@
         <v>30</v>
       </c>
       <c r="H4" s="2">
-        <v>1103</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -996,7 +1026,7 @@
         <v>33</v>
       </c>
       <c r="H5" s="2">
-        <v>2075</v>
+        <v>4187</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1019,21 +1049,21 @@
         <v>33</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H6" s="2">
-        <v>540</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>22</v>
@@ -1042,24 +1072,24 @@
         <v>3</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2">
-        <v>686</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>22</v>
@@ -1068,24 +1098,24 @@
         <v>3</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="H8" s="2">
-        <v>441</v>
+        <v>976</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>22</v>
@@ -1094,24 +1124,24 @@
         <v>3</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H9" s="2">
-        <v>657</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>22</v>
@@ -1120,24 +1150,24 @@
         <v>3</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2">
-        <v>549</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>22</v>
@@ -1146,24 +1176,24 @@
         <v>3</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="H11" s="2">
-        <v>540</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>22</v>
@@ -1172,24 +1202,24 @@
         <v>3</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="H12" s="2">
-        <v>359</v>
+        <v>501</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>22</v>
@@ -1198,24 +1228,24 @@
         <v>3</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H13" s="2">
-        <v>267</v>
+        <v>572</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>22</v>
@@ -1224,24 +1254,24 @@
         <v>3</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="H14" s="2">
-        <v>374</v>
+        <v>533</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>22</v>
@@ -1250,24 +1280,24 @@
         <v>3</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="H15" s="2">
-        <v>312</v>
+        <v>558</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>22</v>
@@ -1276,24 +1306,24 @@
         <v>3</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H16" s="2">
-        <v>336</v>
+        <v>412</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>22</v>
@@ -1302,24 +1332,24 @@
         <v>3</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H17" s="2">
-        <v>318</v>
+        <v>379</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>22</v>
@@ -1328,24 +1358,24 @@
         <v>3</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H18" s="2">
-        <v>303</v>
+        <v>462</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>22</v>
@@ -1354,24 +1384,24 @@
         <v>3</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H19" s="2">
-        <v>503</v>
+        <v>482</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>22</v>
@@ -1386,7 +1416,7 @@
         <v>8</v>
       </c>
       <c r="H20" s="2">
-        <v>295</v>
+        <v>458</v>
       </c>
     </row>
   </sheetData>
@@ -1408,19 +1438,19 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1443,665 +1473,665 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: explicit element wait for Order Success heading before assertions
</commit_message>
<xml_diff>
--- a/excel/E2E_Report.xlsx
+++ b/excel/E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="116">
   <si>
     <t>Execution Date</t>
   </si>
@@ -40,7 +40,7 @@
     <t>Execution Duration (ms)</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:28 AM</t>
+    <t>7/23/2026, 10:30:35 AM</t>
   </si>
   <si>
     <t>Development</t>
@@ -85,10 +85,10 @@
     <t>Chrome</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:03 AM</t>
-  </si>
-  <si>
-    <t>7/23/2026, 10:21:09 AM</t>
+    <t>7/23/2026, 10:30:19 AM</t>
+  </si>
+  <si>
+    <t>7/23/2026, 10:30:22 AM</t>
   </si>
   <si>
     <t>TC-CORE-002</t>
@@ -97,7 +97,7 @@
     <t>Should register a new caterer</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:10 AM</t>
+    <t>7/23/2026, 10:30:24 AM</t>
   </si>
   <si>
     <t>TC-CORE-003</t>
@@ -106,7 +106,7 @@
     <t>Should login as admin and approve the pending caterer</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:12 AM</t>
+    <t>7/23/2026, 10:30:25 AM</t>
   </si>
   <si>
     <t>TC-CORE-004</t>
@@ -115,7 +115,7 @@
     <t>Should login as customer, search, select menu, checkout and confirm booking request</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:16 AM</t>
+    <t>7/23/2026, 10:30:28 AM</t>
   </si>
   <si>
     <t>TC-DYN-001</t>
@@ -127,16 +127,13 @@
     <t>Validate authentication with empty email [TC-DYN-001]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:18 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-002</t>
   </si>
   <si>
     <t>Validate authentication with empty password [TC-DYN-002]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:19 AM</t>
+    <t>7/23/2026, 10:30:29 AM</t>
   </si>
   <si>
     <t>TC-DYN-003</t>
@@ -145,7 +142,7 @@
     <t>Validate authentication with invalid email format [TC-DYN-003]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:20 AM</t>
+    <t>7/23/2026, 10:30:30 AM</t>
   </si>
   <si>
     <t>TC-DYN-004</t>
@@ -154,7 +151,7 @@
     <t>Validate event guest count constraint under min limit (50) [TC-DYN-004]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:22 AM</t>
+    <t>7/23/2026, 10:30:31 AM</t>
   </si>
   <si>
     <t>TC-DYN-005</t>
@@ -163,16 +160,13 @@
     <t>Validate required constraint on field of type number in Checkout [TC-DYN-005]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:23 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-006</t>
   </si>
   <si>
     <t>Validate required constraint on field of type date in Checkout [TC-DYN-006]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:24 AM</t>
+    <t>7/23/2026, 10:30:32 AM</t>
   </si>
   <si>
     <t>TC-DYN-007</t>
@@ -187,7 +181,7 @@
     <t>Validate required constraint on field of type password in Login [TC-DYN-008]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:25 AM</t>
+    <t>7/23/2026, 10:30:33 AM</t>
   </si>
   <si>
     <t>TC-DYN-009</t>
@@ -196,15 +190,15 @@
     <t>Validate required constraint on field of type text in RegisterCaterer [TC-DYN-009]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:26 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-010</t>
   </si>
   <si>
     <t>Validate required constraint on field of type email in RegisterCaterer [TC-DYN-010]</t>
   </si>
   <si>
+    <t>7/23/2026, 10:30:34 AM</t>
+  </si>
+  <si>
     <t>TC-DYN-011</t>
   </si>
   <si>
@@ -217,9 +211,6 @@
     <t>Validate required constraint on field of type password in RegisterCaterer [TC-DYN-012]</t>
   </si>
   <si>
-    <t>7/23/2026, 10:21:27 AM</t>
-  </si>
-  <si>
     <t>TC-DYN-013</t>
   </si>
   <si>
@@ -262,7 +253,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-07-23T04:51:03.556Z</t>
+    <t>2026-07-23T05:00:19.730Z</t>
   </si>
   <si>
     <t>Test Scenario Initiated</t>
@@ -271,7 +262,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-07-23T04:51:09.169Z</t>
+    <t>2026-07-23T05:00:22.321Z</t>
   </si>
   <si>
     <t>Test Scenario Completed</t>
@@ -280,103 +271,97 @@
     <t>Executed successfully</t>
   </si>
   <si>
-    <t>2026-07-23T04:51:09.170Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:10.628Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:10.631Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:12.740Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:12.742Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:16.928Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:16.932Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:18.482Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:18.484Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:19.795Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:19.796Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:20.772Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:20.774Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:22.069Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:22.070Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:23.292Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:23.293Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:24.401Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:24.902Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:24.903Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:25.475Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:26.009Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:26.010Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:26.567Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:26.568Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:26.979Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:27.358Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:27.359Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:27.821Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:27.822Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:28.304Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:28.305Z</t>
-  </si>
-  <si>
-    <t>2026-07-23T04:51:28.762Z</t>
+    <t>2026-07-23T05:00:22.323Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:24.080Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:24.081Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:25.340Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:25.341Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:28.044Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:28.047Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:28.809Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:28.810Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:29.797Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:30.331Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:31.266Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:31.991Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:31.992Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:32.601Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:32.602Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:32.951Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:32.952Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:33.224Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:33.597Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:33.598Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:34.093Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:34.094Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:34.454Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:34.455Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:34.861Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:34.862Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:35.196Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:35.197Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:35.520Z</t>
+  </si>
+  <si>
+    <t>2026-07-23T05:00:35.872Z</t>
   </si>
 </sst>
 </file>
@@ -877,7 +862,7 @@
         <v>10</v>
       </c>
       <c r="H2" s="2">
-        <v>25192</v>
+        <v>16132</v>
       </c>
     </row>
   </sheetData>
@@ -948,7 +933,7 @@
         <v>24</v>
       </c>
       <c r="H2" s="2">
-        <v>5614</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -974,7 +959,7 @@
         <v>27</v>
       </c>
       <c r="H3" s="2">
-        <v>1459</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1000,7 +985,7 @@
         <v>30</v>
       </c>
       <c r="H4" s="2">
-        <v>2111</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1026,7 +1011,7 @@
         <v>33</v>
       </c>
       <c r="H5" s="2">
-        <v>4187</v>
+        <v>2703</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1049,21 +1034,21 @@
         <v>33</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="H6" s="2">
-        <v>1550</v>
+        <v>762</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>22</v>
@@ -1072,24 +1057,24 @@
         <v>3</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H7" s="2">
-        <v>1312</v>
+        <v>988</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>22</v>
@@ -1098,24 +1083,24 @@
         <v>3</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H8" s="2">
-        <v>976</v>
+        <v>534</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>22</v>
@@ -1124,24 +1109,24 @@
         <v>3</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H9" s="2">
-        <v>1296</v>
+        <v>935</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>22</v>
@@ -1150,24 +1135,24 @@
         <v>3</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H10" s="2">
-        <v>1222</v>
+        <v>725</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>22</v>
@@ -1176,24 +1161,24 @@
         <v>3</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H11" s="2">
-        <v>1108</v>
+        <v>609</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>22</v>
@@ -1202,24 +1187,24 @@
         <v>3</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H12" s="2">
-        <v>501</v>
+        <v>350</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>22</v>
@@ -1228,24 +1213,24 @@
         <v>3</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2">
-        <v>572</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>22</v>
@@ -1254,24 +1239,24 @@
         <v>3</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2">
-        <v>533</v>
+        <v>373</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>22</v>
@@ -1280,24 +1265,24 @@
         <v>3</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>60</v>
       </c>
       <c r="H15" s="2">
-        <v>558</v>
+        <v>496</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>22</v>
@@ -1312,18 +1297,18 @@
         <v>60</v>
       </c>
       <c r="H16" s="2">
-        <v>412</v>
+        <v>360</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>22</v>
@@ -1335,21 +1320,21 @@
         <v>60</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="H17" s="2">
-        <v>379</v>
+        <v>406</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>22</v>
@@ -1358,24 +1343,24 @@
         <v>3</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="H18" s="2">
-        <v>462</v>
+        <v>335</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>22</v>
@@ -1384,24 +1369,24 @@
         <v>3</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H19" s="2">
-        <v>482</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>22</v>
@@ -1416,7 +1401,7 @@
         <v>8</v>
       </c>
       <c r="H20" s="2">
-        <v>458</v>
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -1438,19 +1423,19 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1473,665 +1458,665 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>